<commit_message>
feat: update handle import excel file on pxkdl
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/export/MauUploadPCKKVCNB_TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/export/MauUploadPCKKVCNB_TT78.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -34,7 +34,24 @@
     <author>ASIA</author>
   </authors>
   <commentList>
-    <comment ref="V1" authorId="0">
+    <comment ref="Z1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="13"/>
+            <rFont val="Times New Roman"/>
+            <charset val="134"/>
+          </rPr>
+          <t>Tính chất hàng hóa, dịch vụ
+1: HH/DV
+2: KM
+3: GK
+4: Ghi chú</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -56,42 +73,60 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="44">
-  <si>
-    <t>Số phiếu(*)</t>
-  </si>
-  <si>
-    <t>Ngày xuất(*)</t>
-  </si>
-  <si>
-    <t>Lệnh điều động số(*)</t>
-  </si>
-  <si>
-    <t>Người điều động(*)</t>
-  </si>
-  <si>
-    <t>Về việc(*)</t>
-  </si>
-  <si>
-    <t>Người vận chuyển(*)</t>
-  </si>
-  <si>
-    <t>Người xuất hàng</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="47">
+  <si>
+    <t>Mã phiếu(*)</t>
+  </si>
+  <si>
+    <t>Địa chỉ kho xuất hàng (*)</t>
+  </si>
+  <si>
+    <t>Ngày lập (*)</t>
+  </si>
+  <si>
+    <t>Họ và tên người xuất hàng</t>
+  </si>
+  <si>
+    <t>Loại tiền (*)</t>
+  </si>
+  <si>
+    <t>Tên người vận chuyển</t>
   </si>
   <si>
     <t>Hợp đồng số</t>
   </si>
   <si>
-    <t>Phương tiện vận chuyển(*)</t>
-  </si>
-  <si>
-    <t>Xuất tại kho - Mã kho(*)</t>
-  </si>
-  <si>
-    <t>Nhập tại kho - Mã kho(*)</t>
-  </si>
-  <si>
-    <t>Email nhận</t>
+    <t>Lệnh điều động nội bộ (*)</t>
+  </si>
+  <si>
+    <t>Phương tiện vận chuyển (*)</t>
+  </si>
+  <si>
+    <t>Mã số thuế người nhập</t>
+  </si>
+  <si>
+    <t>Họ và Tên người nhập</t>
+  </si>
+  <si>
+    <t>Tên đơn vị nhập</t>
+  </si>
+  <si>
+    <t>Địa chỉ kho nhập hàng(*)</t>
+  </si>
+  <si>
+    <t>Nội dung nhập kho</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Số điện thoại</t>
+  </si>
+  <si>
+    <t>Số tài khoản</t>
+  </si>
+  <si>
+    <t>Tại ngân hàng</t>
   </si>
   <si>
     <t>STT(*)</t>
@@ -106,10 +141,7 @@
     <t>Đơn vị tính</t>
   </si>
   <si>
-    <t>Thực xuất(*)</t>
-  </si>
-  <si>
-    <t>Thực nhập</t>
+    <t>Số lượng(*)</t>
   </si>
   <si>
     <t>Đơn giá(*)</t>
@@ -118,43 +150,31 @@
     <t>Thành tiền(*)</t>
   </si>
   <si>
-    <t>Tổng tiền(*)</t>
-  </si>
-  <si>
     <t>Tính Chất(*)</t>
   </si>
   <si>
-    <t>Số tiền bằng chữ</t>
+    <t>Tỷ giá(*)</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>05/06/2022</t>
-  </si>
-  <si>
-    <t>DD001</t>
-  </si>
-  <si>
-    <t>Nguyen Văn A</t>
-  </si>
-  <si>
-    <t>Chuyển kho</t>
-  </si>
-  <si>
-    <t>Nguyen Van C</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Xe tải</t>
-  </si>
-  <si>
-    <t>WH01</t>
-  </si>
-  <si>
-    <t>WH02</t>
+    <t>Địa chỉ xuất kho 1</t>
+  </si>
+  <si>
+    <t>12/05/2026</t>
+  </si>
+  <si>
+    <t>VND</t>
+  </si>
+  <si>
+    <t>01002/HĐKG/2026</t>
+  </si>
+  <si>
+    <t>Xe</t>
+  </si>
+  <si>
+    <t>Địa chỉ kho nhập 1</t>
   </si>
   <si>
     <t>sản phẩm 1</t>
@@ -166,25 +186,31 @@
     <t>CAI</t>
   </si>
   <si>
+    <t>200000</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
     <t>sản phẩm 2</t>
   </si>
   <si>
-    <t>Nguyen Văn B</t>
-  </si>
-  <si>
-    <t>Nguyen Van D</t>
-  </si>
-  <si>
-    <t>xxx@gmail.com</t>
+    <t>100000</t>
+  </si>
+  <si>
+    <t>Tàu</t>
+  </si>
+  <si>
+    <t>Địa chỉ kho nhập 2</t>
   </si>
   <si>
     <t>sp1</t>
   </si>
   <si>
     <t>gói</t>
+  </si>
+  <si>
+    <t>50000</t>
   </si>
   <si>
     <t>END</t>
@@ -200,7 +226,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,12 +243,12 @@
     </font>
     <font>
       <sz val="13"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="13"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
@@ -241,11 +267,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -390,7 +428,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -405,7 +443,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor theme="9" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -580,12 +618,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -726,175 +758,199 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -903,12 +959,12 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1243,255 +1299,1126 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:W5"/>
-  <sheetFormatPr defaultColWidth="25.4285714285714" defaultRowHeight="16.5" outlineLevelRow="4"/>
+  <dimension ref="A1:AA33"/>
+  <sheetFormatPr defaultColWidth="25.4571428571429" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="8" width="25.4285714285714" style="2"/>
-    <col min="9" max="9" width="30.8571428571429" style="2" customWidth="1"/>
-    <col min="10" max="10" width="29.4285714285714" style="2" customWidth="1"/>
-    <col min="11" max="11" width="29.1428571428571" style="2" customWidth="1"/>
-    <col min="12" max="16" width="25.4285714285714" style="2"/>
-    <col min="17" max="21" width="25.4285714285714" style="3"/>
-    <col min="22" max="22" width="25.4285714285714" style="4"/>
-    <col min="23" max="23" width="25.4285714285714" style="3"/>
-    <col min="24" max="16384" width="25.4285714285714" style="5"/>
+    <col min="1" max="1" width="25.4571428571429" style="3"/>
+    <col min="2" max="2" width="40.5714285714286" style="3" customWidth="1"/>
+    <col min="3" max="3" width="25.4571428571429" style="4"/>
+    <col min="4" max="4" width="33.7142857142857" style="3" customWidth="1"/>
+    <col min="5" max="5" width="25.4571428571429" style="4"/>
+    <col min="6" max="6" width="29.8571428571429" style="3" customWidth="1"/>
+    <col min="7" max="7" width="28" style="3" customWidth="1"/>
+    <col min="8" max="8" width="30.8571428571429" style="4" customWidth="1"/>
+    <col min="9" max="9" width="32.4285714285714" style="3" customWidth="1"/>
+    <col min="10" max="10" width="27.1428571428571" style="3" customWidth="1"/>
+    <col min="11" max="12" width="25.4571428571429" style="3"/>
+    <col min="13" max="13" width="29.8571428571429" style="3" customWidth="1"/>
+    <col min="14" max="22" width="25.4571428571429" style="3"/>
+    <col min="23" max="26" width="25.4571428571429" style="5"/>
+    <col min="27" max="27" width="25.4571428571429" style="6"/>
+    <col min="28" max="16384" width="25.4571428571429" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:23">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="1" customFormat="1" spans="1:27">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="8" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="P1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="R1" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="W1" s="12" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:22">
-      <c r="A2" s="12" t="s">
+      <c r="X1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="Y1" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="Z1" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="AA1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="2" t="s">
+    </row>
+    <row r="2" s="2" customFormat="1" spans="1:27">
+      <c r="A2" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N2" s="2" t="s">
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="N2" s="3"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="T2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="U2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="V2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="W2" s="5">
         <v>1</v>
       </c>
-      <c r="S2" s="3">
-        <v>0</v>
-      </c>
-      <c r="T2" s="3">
-        <f t="shared" ref="T2:T3" si="0">Q2*S2</f>
-        <v>0</v>
-      </c>
-      <c r="U2" s="3">
-        <v>0</v>
-      </c>
-      <c r="V2" s="4">
+      <c r="X2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y2" s="5">
+        <f>W2*X2</f>
+        <v>200000</v>
+      </c>
+      <c r="Z2" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:22">
-      <c r="A3" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" s="2" t="s">
+      <c r="AA2" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" s="2" customFormat="1" spans="1:27">
+      <c r="A3" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="V3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="N3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q3" s="3">
+      <c r="W3" s="5">
         <v>2</v>
       </c>
-      <c r="S3" s="3">
-        <v>0</v>
-      </c>
-      <c r="T3" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="U3" s="3">
-        <v>0</v>
-      </c>
-      <c r="V3" s="4">
+      <c r="X3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y3" s="5">
+        <f>W3*X3</f>
+        <v>200000</v>
+      </c>
+      <c r="Z3" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:22">
-      <c r="A4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="AA3" s="6"/>
+    </row>
+    <row r="4" s="2" customFormat="1" spans="1:27">
+      <c r="A4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="N4" s="3"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L4" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="P4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q4" s="3">
+      <c r="T4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="W4" s="5">
         <v>12</v>
       </c>
-      <c r="S4" s="3">
-        <v>0</v>
-      </c>
-      <c r="T4" s="3">
-        <v>0</v>
-      </c>
-      <c r="U4" s="3">
-        <v>0</v>
-      </c>
-      <c r="V4" s="4">
+      <c r="X4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4" s="5">
+        <f>W4*X4</f>
+        <v>600000</v>
+      </c>
+      <c r="Z4" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="AA4" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" s="2" customFormat="1" spans="1:27">
+      <c r="A5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
+      <c r="S5" s="16"/>
+      <c r="T5" s="16"/>
+      <c r="U5" s="16"/>
+      <c r="V5" s="16"/>
+      <c r="W5" s="18"/>
+      <c r="X5" s="18"/>
+      <c r="Y5" s="18"/>
+      <c r="Z5" s="18"/>
+      <c r="AA5" s="19"/>
+    </row>
+    <row r="6" spans="1:27">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="S6" s="16"/>
+      <c r="T6" s="16"/>
+      <c r="U6" s="16"/>
+      <c r="V6" s="16"/>
+      <c r="W6" s="18"/>
+      <c r="X6" s="18"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="18"/>
+      <c r="AA6" s="19"/>
+    </row>
+    <row r="7" spans="1:27">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16"/>
+      <c r="W7" s="18"/>
+      <c r="X7" s="18"/>
+      <c r="Y7" s="18"/>
+      <c r="Z7" s="18"/>
+      <c r="AA7" s="19"/>
+    </row>
+    <row r="8" spans="1:27">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
+      <c r="P8" s="16"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="16"/>
+      <c r="V8" s="16"/>
+      <c r="W8" s="18"/>
+      <c r="X8" s="18"/>
+      <c r="Y8" s="18"/>
+      <c r="Z8" s="18"/>
+      <c r="AA8" s="19"/>
+    </row>
+    <row r="9" spans="1:27">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="16"/>
+      <c r="U9" s="16"/>
+      <c r="V9" s="16"/>
+      <c r="W9" s="18"/>
+      <c r="X9" s="18"/>
+      <c r="Y9" s="18"/>
+      <c r="Z9" s="18"/>
+      <c r="AA9" s="19"/>
+    </row>
+    <row r="10" spans="1:27">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="16"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+      <c r="V10" s="16"/>
+      <c r="W10" s="18"/>
+      <c r="X10" s="18"/>
+      <c r="Y10" s="18"/>
+      <c r="Z10" s="18"/>
+      <c r="AA10" s="19"/>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="16"/>
+      <c r="Q11" s="16"/>
+      <c r="R11" s="16"/>
+      <c r="S11" s="16"/>
+      <c r="T11" s="16"/>
+      <c r="U11" s="16"/>
+      <c r="V11" s="16"/>
+      <c r="W11" s="18"/>
+      <c r="X11" s="18"/>
+      <c r="Y11" s="18"/>
+      <c r="Z11" s="18"/>
+      <c r="AA11" s="19"/>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="16"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
+      <c r="S12" s="16"/>
+      <c r="T12" s="16"/>
+      <c r="U12" s="16"/>
+      <c r="V12" s="16"/>
+      <c r="W12" s="18"/>
+      <c r="X12" s="18"/>
+      <c r="Y12" s="18"/>
+      <c r="Z12" s="18"/>
+      <c r="AA12" s="19"/>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="16"/>
+      <c r="O13" s="16"/>
+      <c r="P13" s="16"/>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="16"/>
+      <c r="S13" s="16"/>
+      <c r="T13" s="16"/>
+      <c r="U13" s="16"/>
+      <c r="V13" s="16"/>
+      <c r="W13" s="18"/>
+      <c r="X13" s="18"/>
+      <c r="Y13" s="18"/>
+      <c r="Z13" s="18"/>
+      <c r="AA13" s="19"/>
+    </row>
+    <row r="14" spans="1:27">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="16"/>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
+      <c r="S14" s="16"/>
+      <c r="T14" s="16"/>
+      <c r="U14" s="16"/>
+      <c r="V14" s="16"/>
+      <c r="W14" s="18"/>
+      <c r="X14" s="18"/>
+      <c r="Y14" s="18"/>
+      <c r="Z14" s="18"/>
+      <c r="AA14" s="19"/>
+    </row>
+    <row r="15" spans="1:27">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16"/>
+      <c r="P15" s="16"/>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="16"/>
+      <c r="S15" s="16"/>
+      <c r="T15" s="16"/>
+      <c r="U15" s="16"/>
+      <c r="V15" s="16"/>
+      <c r="W15" s="18"/>
+      <c r="X15" s="18"/>
+      <c r="Y15" s="18"/>
+      <c r="Z15" s="18"/>
+      <c r="AA15" s="19"/>
+    </row>
+    <row r="16" spans="1:27">
+      <c r="A16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="16"/>
+      <c r="U16" s="16"/>
+      <c r="V16" s="16"/>
+      <c r="W16" s="18"/>
+      <c r="X16" s="18"/>
+      <c r="Y16" s="18"/>
+      <c r="Z16" s="18"/>
+      <c r="AA16" s="19"/>
+    </row>
+    <row r="17" spans="1:27">
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
+      <c r="S17" s="16"/>
+      <c r="T17" s="16"/>
+      <c r="U17" s="16"/>
+      <c r="V17" s="16"/>
+      <c r="W17" s="18"/>
+      <c r="X17" s="18"/>
+      <c r="Y17" s="18"/>
+      <c r="Z17" s="18"/>
+      <c r="AA17" s="19"/>
+    </row>
+    <row r="18" spans="1:27">
+      <c r="A18" s="16"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
+      <c r="U18" s="16"/>
+      <c r="V18" s="16"/>
+      <c r="W18" s="18"/>
+      <c r="X18" s="18"/>
+      <c r="Y18" s="18"/>
+      <c r="Z18" s="18"/>
+      <c r="AA18" s="19"/>
+    </row>
+    <row r="19" spans="1:27">
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
+      <c r="S19" s="16"/>
+      <c r="T19" s="16"/>
+      <c r="U19" s="16"/>
+      <c r="V19" s="16"/>
+      <c r="W19" s="18"/>
+      <c r="X19" s="18"/>
+      <c r="Y19" s="18"/>
+      <c r="Z19" s="18"/>
+      <c r="AA19" s="19"/>
+    </row>
+    <row r="20" spans="1:27">
+      <c r="A20" s="16"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
+      <c r="S20" s="16"/>
+      <c r="T20" s="16"/>
+      <c r="U20" s="16"/>
+      <c r="V20" s="16"/>
+      <c r="W20" s="18"/>
+      <c r="X20" s="18"/>
+      <c r="Y20" s="18"/>
+      <c r="Z20" s="18"/>
+      <c r="AA20" s="19"/>
+    </row>
+    <row r="21" spans="1:27">
+      <c r="A21" s="16"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="16"/>
+      <c r="T21" s="16"/>
+      <c r="U21" s="16"/>
+      <c r="V21" s="16"/>
+      <c r="W21" s="18"/>
+      <c r="X21" s="18"/>
+      <c r="Y21" s="18"/>
+      <c r="Z21" s="18"/>
+      <c r="AA21" s="19"/>
+    </row>
+    <row r="22" spans="1:27">
+      <c r="A22" s="16"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="S22" s="16"/>
+      <c r="T22" s="16"/>
+      <c r="U22" s="16"/>
+      <c r="V22" s="16"/>
+      <c r="W22" s="18"/>
+      <c r="X22" s="18"/>
+      <c r="Y22" s="18"/>
+      <c r="Z22" s="18"/>
+      <c r="AA22" s="19"/>
+    </row>
+    <row r="23" spans="1:27">
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="16"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="16"/>
+      <c r="T23" s="16"/>
+      <c r="U23" s="16"/>
+      <c r="V23" s="16"/>
+      <c r="W23" s="18"/>
+      <c r="X23" s="18"/>
+      <c r="Y23" s="18"/>
+      <c r="Z23" s="18"/>
+      <c r="AA23" s="19"/>
+    </row>
+    <row r="24" spans="1:27">
+      <c r="A24" s="16"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16"/>
+      <c r="M24" s="16"/>
+      <c r="N24" s="16"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="S24" s="16"/>
+      <c r="T24" s="16"/>
+      <c r="U24" s="16"/>
+      <c r="V24" s="16"/>
+      <c r="W24" s="18"/>
+      <c r="X24" s="18"/>
+      <c r="Y24" s="18"/>
+      <c r="Z24" s="18"/>
+      <c r="AA24" s="19"/>
+    </row>
+    <row r="25" spans="1:27">
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="16"/>
+      <c r="N25" s="16"/>
+      <c r="O25" s="16"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="16"/>
+      <c r="T25" s="16"/>
+      <c r="U25" s="16"/>
+      <c r="V25" s="16"/>
+      <c r="W25" s="18"/>
+      <c r="X25" s="18"/>
+      <c r="Y25" s="18"/>
+      <c r="Z25" s="18"/>
+      <c r="AA25" s="19"/>
+    </row>
+    <row r="26" spans="1:27">
+      <c r="A26" s="16"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="16"/>
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="16"/>
+      <c r="T26" s="16"/>
+      <c r="U26" s="16"/>
+      <c r="V26" s="16"/>
+      <c r="W26" s="18"/>
+      <c r="X26" s="18"/>
+      <c r="Y26" s="18"/>
+      <c r="Z26" s="18"/>
+      <c r="AA26" s="19"/>
+    </row>
+    <row r="27" spans="1:27">
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="16"/>
+      <c r="T27" s="16"/>
+      <c r="U27" s="16"/>
+      <c r="V27" s="16"/>
+      <c r="W27" s="18"/>
+      <c r="X27" s="18"/>
+      <c r="Y27" s="18"/>
+      <c r="Z27" s="18"/>
+      <c r="AA27" s="19"/>
+    </row>
+    <row r="28" spans="1:27">
+      <c r="A28" s="16"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="16"/>
+      <c r="T28" s="16"/>
+      <c r="U28" s="16"/>
+      <c r="V28" s="16"/>
+      <c r="W28" s="18"/>
+      <c r="X28" s="18"/>
+      <c r="Y28" s="18"/>
+      <c r="Z28" s="18"/>
+      <c r="AA28" s="19"/>
+    </row>
+    <row r="29" spans="1:27">
+      <c r="A29" s="16"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="16"/>
+      <c r="L29" s="16"/>
+      <c r="M29" s="16"/>
+      <c r="N29" s="16"/>
+      <c r="O29" s="16"/>
+      <c r="P29" s="16"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
+      <c r="S29" s="16"/>
+      <c r="T29" s="16"/>
+      <c r="U29" s="16"/>
+      <c r="V29" s="16"/>
+      <c r="W29" s="18"/>
+      <c r="X29" s="18"/>
+      <c r="Y29" s="18"/>
+      <c r="Z29" s="18"/>
+      <c r="AA29" s="19"/>
+    </row>
+    <row r="30" spans="1:27">
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="16"/>
+      <c r="N30" s="16"/>
+      <c r="O30" s="16"/>
+      <c r="P30" s="16"/>
+      <c r="Q30" s="16"/>
+      <c r="R30" s="16"/>
+      <c r="S30" s="16"/>
+      <c r="T30" s="16"/>
+      <c r="U30" s="16"/>
+      <c r="V30" s="16"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="18"/>
+      <c r="Z30" s="18"/>
+      <c r="AA30" s="19"/>
+    </row>
+    <row r="31" spans="1:27">
+      <c r="A31" s="16"/>
+      <c r="B31" s="16"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
+      <c r="M31" s="16"/>
+      <c r="N31" s="16"/>
+      <c r="O31" s="16"/>
+      <c r="P31" s="16"/>
+      <c r="Q31" s="16"/>
+      <c r="R31" s="16"/>
+      <c r="S31" s="16"/>
+      <c r="T31" s="16"/>
+      <c r="U31" s="16"/>
+      <c r="V31" s="16"/>
+      <c r="W31" s="18"/>
+      <c r="X31" s="18"/>
+      <c r="Y31" s="18"/>
+      <c r="Z31" s="18"/>
+      <c r="AA31" s="19"/>
+    </row>
+    <row r="32" spans="1:27">
+      <c r="A32" s="16"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="16"/>
+      <c r="M32" s="16"/>
+      <c r="N32" s="16"/>
+      <c r="O32" s="16"/>
+      <c r="P32" s="16"/>
+      <c r="Q32" s="16"/>
+      <c r="R32" s="16"/>
+      <c r="S32" s="16"/>
+      <c r="T32" s="16"/>
+      <c r="U32" s="16"/>
+      <c r="V32" s="16"/>
+      <c r="W32" s="18"/>
+      <c r="X32" s="18"/>
+      <c r="Y32" s="18"/>
+      <c r="Z32" s="18"/>
+      <c r="AA32" s="19"/>
+    </row>
+    <row r="33" spans="1:27">
+      <c r="A33" s="16"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="16"/>
+      <c r="L33" s="16"/>
+      <c r="M33" s="16"/>
+      <c r="N33" s="16"/>
+      <c r="O33" s="16"/>
+      <c r="P33" s="16"/>
+      <c r="Q33" s="16"/>
+      <c r="R33" s="16"/>
+      <c r="S33" s="16"/>
+      <c r="T33" s="16"/>
+      <c r="U33" s="16"/>
+      <c r="V33" s="16"/>
+      <c r="W33" s="18"/>
+      <c r="X33" s="18"/>
+      <c r="Y33" s="18"/>
+      <c r="Z33" s="18"/>
+      <c r="AA33" s="19"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="L4" r:id="rId3" display="xxx@gmail.com"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>
   <headerFooter/>

</xml_diff>